<commit_message>
BETA 0.9.9: corrige M.O.D (quantidade na coluna G), campo OS em 2 linhas, refresh de sessao (Funcao/Perfil), limpar dados salvos completo
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/modelo_rdo.xlsx
+++ b/assets/modelo_rdo.xlsx
@@ -192,10 +192,11 @@
 </t>
   </si>
   <si>
-    <t>OS:                 XXXX</t>
-  </si>
-  <si>
-    <t>Modelo V.1.3</t>
+    <t xml:space="preserve">OS:
+</t>
+  </si>
+  <si>
+    <t>Modelo V.1.4</t>
   </si>
   <si>
     <t>XXXX-AAAAMMDD</t>

</xml_diff>